<commit_message>
perfect for 1st Phase Release
</commit_message>
<xml_diff>
--- a/Tirap_Performance_Index_v2 Updated.xlsx
+++ b/Tirap_Performance_Index_v2 Updated.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8196" tabRatio="500" firstSheet="13" activeTab="14"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8196" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Cover &amp; Instructions" sheetId="1" r:id="rId1"/>
@@ -9799,7 +9799,7 @@
       </c>
       <c r="B2" s="63"/>
       <c r="C2" s="7" t="s">
-        <v>115</v>
+        <v>55</v>
       </c>
       <c r="D2" s="64" t="s">
         <v>56</v>

</xml_diff>